<commit_message>
Sequences are close to be done
</commit_message>
<xml_diff>
--- a/Gudeline 36 data.xlsx
+++ b/Gudeline 36 data.xlsx
@@ -1,32 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git Projects\PsychroCalc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB08FEDB-E5A2-492F-BF42-3A2D0B2C3190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C594318-14C2-401D-A2AC-D969760C1A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setpoints_Requirements" sheetId="1" r:id="rId1"/>
     <sheet name="Points_Lists" sheetId="2" r:id="rId2"/>
     <sheet name="Sequences" sheetId="3" r:id="rId3"/>
     <sheet name="Tables" sheetId="4" r:id="rId4"/>
+    <sheet name="Logic" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_Ref38822284" localSheetId="2">Sequences!$A$126</definedName>
-    <definedName name="_Ref440033356" localSheetId="2">Sequences!$D$19</definedName>
-    <definedName name="_Ref73449741" localSheetId="2">Sequences!$A$30</definedName>
-    <definedName name="_Ref73449755" localSheetId="2">Sequences!$A$29</definedName>
-    <definedName name="_Ref73450375" localSheetId="2">Sequences!$A$40</definedName>
-    <definedName name="_Ref73450525" localSheetId="2">Sequences!$A$51</definedName>
-    <definedName name="_Ref73451565" localSheetId="2">Sequences!$A$95</definedName>
-    <definedName name="_Ref73451586" localSheetId="2">Sequences!$A$291</definedName>
+    <definedName name="_Ref38822284" localSheetId="2">Sequences!$A$134</definedName>
+    <definedName name="_Ref440015150" localSheetId="2">Sequences!$G$12</definedName>
+    <definedName name="_Ref440015169" localSheetId="2">Sequences!$G$11</definedName>
+    <definedName name="_Ref440033356" localSheetId="2">Sequences!$D$27</definedName>
+    <definedName name="_Ref73449741" localSheetId="2">Sequences!$A$38</definedName>
+    <definedName name="_Ref73449755" localSheetId="2">Sequences!$A$37</definedName>
+    <definedName name="_Ref73450375" localSheetId="2">Sequences!$A$48</definedName>
+    <definedName name="_Ref73450525" localSheetId="2">Sequences!$A$59</definedName>
+    <definedName name="_Ref73451565" localSheetId="2">Sequences!$A$103</definedName>
+    <definedName name="_Ref73451586" localSheetId="2">Sequences!$A$299</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="284">
   <si>
     <t>Design Requirements Table</t>
   </si>
@@ -648,16 +651,6 @@
     <t>Trim_and_Respond_Table</t>
   </si>
   <si>
-    <t>Supply Fan Start/Stop
-a.	Supply fan shall run when system is in the Cooldown Mode, Setup Mode, or Occupied Mode.
-b.	If there are any VAV-reheat boxes on perimeter zones, supply fan shall also run when system is in Setback Mode or Warmup Mode (i.e., all modes except unoccupied).
-c.	Totalize current airflow rate from VAV boxes to a software point Vps. 
-5.16.1.2.	Static Pressure Set-Point Reset
-a.	Static pressure setpoint. Setpoint shall be reset using T&amp;R logic (see Section 5.1.14 from ASHRAE guideline 36) using the parameters shown in trim and respond table. 
-Static Pressure Control
-a.	Supply fan speed is controlled to maintain DSP at setpoint when the fan is proven ON. Where the Zone Groups served by the system are small, provide multiple sets of gains that are used in the control loop as a function of a load indicator (such as supply-fan airflow rate, the area of the Zone Groups that are occupied, etc.).</t>
-  </si>
-  <si>
     <t>Static Pressure</t>
   </si>
   <si>
@@ -748,33 +741,18 @@
     <t>Section Applicable if</t>
   </si>
   <si>
-    <t>Applicable</t>
-  </si>
-  <si>
     <t>yes</t>
-  </si>
-  <si>
-    <t>Retun fan</t>
   </si>
   <si>
     <t>b.	For units with relief dampers or relief fans
 1.	Economizer damper minimum position MinOA-P and/or return air damper maximum position MaxRA-P are modulated to control minimum outdoor air volume (see Sections related to minimum outdoor air control).</t>
   </si>
   <si>
-    <t>Saperate min OA and Econ Damper</t>
-  </si>
-  <si>
-    <t>2.	For units with a separate minimum outdoor air damper, economizer damper minimum position MinOA-P is 0%, and return air damper maximum position MaxRA-P is modulated to control minimum outdoor air volume (see Sections related to minimum outdoor air control).</t>
-  </si>
-  <si>
-    <t>Single Econ and OA damper</t>
-  </si>
-  <si>
-    <t>2.	For units with a single common minimum outdoor air and economizer damper, return air damper maximum position MaxRA-P and economizer damper minimum position MinOA-P are modulated to control minimum outdoor air volume (see Section 5.16.6). Economizer damper maximum position MaxOA-P is limited during minimum outdoor air control (e.g., economizer lockout due to high OAT).</t>
-  </si>
-  <si>
     <t>b.	For units with return fans
 1.	Return air damper maximum position MaxRA-P is modulated to control minimum outdoor air volume (see Sections related to minimum outdoor air control).</t>
+  </si>
+  <si>
+    <t>ahsrae 62.1</t>
   </si>
   <si>
     <t>Control loop is enabled when the supply air fan is proven ON, and disabled and output set to deadband (no heating, minimum economizer) otherwise.
@@ -785,13 +763,276 @@
 c.	During Cooldown Mode, setpoint shall be Min_ClgSAT.
 d.	During Warmup Mode and Setback Mode, setpoint shall be 35°C (95°F).
 2.            Supply air temperature shall be controlled to setpoint using a control loop whose output is mapped to sequence the heating coil (if applicable), outdoor air damper, return air damper, and cooling coil as shown in Figure shown. 
-a.	The points of transition along the x-axis shown and described in Figures are representative. Separate gains shall be provided for each section of the control map (heating coil, economizer, cooling coil) that is determined by the contractor to provide stable control. Alternatively, the contractor shall adjust the precise value of the x-axis thresholds shown in Figure to provide stable control. Damper control depends on the type of building pressure control system.</t>
-  </si>
-  <si>
-    <t>ahsrae 62.1</t>
+a.	The points of transition along the x-axis shown and described in Figures in ASHRAE Guideline 36 are representative. Separate gains shall be provided for each section of the control map (heating coil, economizer, cooling coil) that is determined by the contractor to provide stable control. Alternatively, the contractor shall adjust the precise value of the x-axis thresholds shown in Figure to provide stable control. Damper control depends on the type of building pressure control system.</t>
+  </si>
+  <si>
+    <t>VAV SEQUENCE STEPS</t>
+  </si>
+  <si>
+    <t>supply fan control</t>
+  </si>
+  <si>
+    <t>Supply air temp control</t>
+  </si>
+  <si>
+    <t>If return fan</t>
+  </si>
+  <si>
+    <t>If relief fan</t>
+  </si>
+  <si>
+    <t>If saperate min oa and econ damper</t>
+  </si>
+  <si>
+    <t>if single oa damper</t>
+  </si>
+  <si>
+    <t>Minimum OA Setpoint</t>
+  </si>
+  <si>
+    <t>If Ashrae 62.1</t>
+  </si>
+  <si>
+    <t>If Title 24</t>
+  </si>
+  <si>
+    <t>Ashrae 62.1</t>
+  </si>
+  <si>
+    <t>single_damper</t>
+  </si>
+  <si>
+    <t>min_and_econ_damper</t>
+  </si>
+  <si>
+    <t>min_and_econ_damper_62.1</t>
+  </si>
+  <si>
+    <t>min_and_econ_damper_24</t>
+  </si>
+  <si>
+    <t>single_damper_62.1</t>
+  </si>
+  <si>
+    <t>single_damper_24</t>
+  </si>
+  <si>
+    <t>OA and RA Damper</t>
+  </si>
+  <si>
+    <t>Outdoor Air and Return Air Dampers</t>
+  </si>
+  <si>
+    <t>min_and_econ_damper_Rreturnfan</t>
+  </si>
+  <si>
+    <t>a.	For units with return fans
+1.	When the supply air fan is proven on and the system is in Occupied Mode and MinOAsp is greater than zero, the system shall calculate MRA-P.  The value of MRA-P shall scale from 95% when supply fan speed is at 100% design speed proportionally down to 20% when the fan is at minimum speed.  When MRA-P is not being calculated for any reason, it shall be set to 100%.
+2.	Minimum outdoor air control shall be enabled when the unit is in Occupied Mode and either of the following conditions are true for 10 minutes:
+i.	The economizer high limit conditions in Section 5.1.17 are exceeded.
+ii.	When the minimum outdoor air damper is open and the return air damper position is greater than MRA-P.
+3.	When minimum outdoor air control is enabled, the normal sequencing of economizer outdoor air and return air dampers per Section 5.16.2 shall be suspended per the following sequence:
+i.	Fully open return air damper; and
+ii.	Wait 15 seconds, then close the economizer outdoor air damper; and
+iii.	Wait 3 minutes, then release return air damper position for control by the SAT control loop in Section 5.16.2.  Economizer outdoor air damper remains closed.
+iv.	The maximum return air damper position endpoint MaxRA-P shall be modulated from 100% to 0% to maintain airflow across the minimum outdoor air damper at setpoint MinOAsp.
+4.	Minimum outdoor air control shall be disabled when the unit is no longer in Occupied Mode, or both of the following conditions are true for 10 minutes:
+i.	The economizer high limit conditions in Section 5.1.17 are exceeded.
+ii.	The minimum outdoor air damper is closed or the return air damper position is 10% below MRA-P.
+5.	When minimum outdoor air control is disabled:
+i.	Economizer outdoor air damper shall be fully opened.
+ii.	MaxRA-P shall be set to 100%.
+iii.	Economizer and return air damper positions shall be controlled by the SAT control loop per Section 5.16.2.</t>
+  </si>
+  <si>
+    <t>min_and_econ_damper_relieffan</t>
+  </si>
+  <si>
+    <t>a.	For units with relief dampers or relief fans
+1.	When the supply air fan is proven on and the system is in occupied mode and MinOAsp is greater than zero, the system shall calculate MOA-P.  The value of MOA-P shall scale from 5% when supply-fan speed is at 100% design speed proportionally up to 80% when the fan is at minimum speed.  When MOA-P is not being calculated for any reason, it shall be set to 0%.
+2.	When the supply air fan is proven on and the system is in occupied mode and MinOAsp is greater than zero, the system shall calculate MRA-P.  The value of MRA-P shall scale from 95% when supply fan speed is at 100% design speed proportionally down to 20% when the fan is at minimum speed.  When MRA-P is not being calculated for any reason, it shall be set to 100%.
+3.	Minimum outdoor air control shall be enabled when the unit is in Occupied Mode and either of the following conditions are true for 10 minutes:
+i.	The economizer high limit conditions in Section 5.1.17 are exceeded.
+ii.	When the minimum outdoor air damper is open and the economizer outdoor air damper position is less than MOA-P.
+4.	When minimum outdoor air control is enabled, the normal sequencing of economizer outdoor air and return air dampers per Section 5.16.2 shall be superseded per the following:
+i.	Fully open return air damper; and 
+ii.	Wait 15 seconds, then close the economizer outdoor air damper; and
+iii.	Wait 3 minutes, then release return air damper position for control by the SAT control loop in Section 5.16.2.  Economizer outdoor air damper remains closed.
+iv.	The maximum return air damper position endpoint MaxRA-P shall be modulated from 100% to 0% to maintain airflow across the minimum outdoor air damper at setpoint MinOAsp.
+5.	Minimum outdoor air control shall be disabled when the unit is no longer in Occupied Mode, or both of the following conditions are true for 10 minutes:
+i.	The economizer high limit conditions in Section 5.1.17 are not exceeded.
+ii.	The minimum outdoor air damper is closed or the return air damper position is 10% below MRA-P.
+6.	When minimum outdoor air control is disabled:
+i.	MaxRA-P shall be set to 100%.
+ii.	Economizer and return air damper positions shall be controlled by the SAT control loop per Section 5.16.2.</t>
+  </si>
+  <si>
+    <t>single_damper_relieffan</t>
+  </si>
+  <si>
+    <t>single_damper_returnfan</t>
+  </si>
+  <si>
+    <t>Outdoor Airflow Setpoint for ASHRAE Standard 62.1-2016 Ventilation
+a.	See Section 5.16.3.1 for calculation of current outdoor air setpoint MinOAsp.
+Minimum Outdoor Air Control Loop
+a.	Minimum outdoor air control loop is enabled when the supply fan is proven ON and the AHU is in Occupied Mode, and disabled and output set to zero otherwise.</t>
   </si>
   <si>
     <t>Outdoor Airflow Setpoint for California Title 24 Ventilation
+a.	See Section 5.16.3.2 for calculation of current setpoints AbsMinOA* and DesMinOA*.
+b.	See zone CO2 control logic under terminal unit sequences.
+c.	The minimum outdoor air setpoint MinOAsp shall be reset based on the highest zone CO2 control-loop signal from AbsMinOA* at 50% signal to DesMinOA* at 100% signal.
+Minimum Outdoor Air Control Loop
+a.	Minimum outdoor air control loop is enabled when the supply fan is proven ON and the AHU is in Occupied Mode, and disabled and output set to zero otherwise.</t>
+  </si>
+  <si>
+    <t>For units with return fans:
+1.	The outdoor airflow rate shall be maintained at the minimum outdoor damper outdoor airflow setpoint MinOAsp by a direct-acting control loop whose output is mapped to the return air damper maximum position endpoint MaxRA-P.
+2.	While the unit is in Occupied Mode, if the economizer high limit conditions in Section 5.1.17 are exceeded for 10 minutes, outdoor air shall be controlled to the minimum outdoor airflow.  When this occurs, the normal sequencing of the return air damper by the SAT control loop is suspended, and the return air damper position shall be modulated directly to maintain measured airflow at MinOAsp (i.e. return damper position shall equal MaxRA-P).  The economizer damper shall remain open.
+3.	If the economizer high limit conditions in Section 5.1.17 are not exceeded for 10 minutes, or the unit is no longer in Occupied Mode, release return damper to control by the SAT control loop (i.e. return damper position is limited by MaxRA-P endpoint, but is not directly controlled to equal MaxRA-P).</t>
+  </si>
+  <si>
+    <t>For units with relief dampers or relief fans:
+1.	The outdoor airflow rate shall be maintained at the minimum outdoor air setpoint MinOAsp by a reverse-acting control loop whose output is mapped to economizer damper minimum position MinOA-P and return air damper maximum position MaxRA-P as indicated in Figure 5.16.6.3.
+2.	While the unit is in Occupied Mode, if the economizer high limit conditions in Section 5.1.17 are exceeded for 10 minutes, outdoor airflow shall be controlled to the minimum outdoor airflow setpoint, MinOAsp.  When this occurs, the normal sequencing of the return air damper by the SAT control loop is suspended as follows:
+i.	Fully open the return air damper
+ii.	Wait 15 seconds, then set MaxOA-P equal to MinOA-P
+iii.	Wait 3 minutes, then modulate the return air damper to maintain the measured airflow at MinOAsp (i.e. return air damper position shall equal MaxRA-P).
+3.	If the economizer high limit conditions in Section 5.1.17 are not exceeded for 10 minutes, or the unit is no longer in Occupied Mode, set MaxOA-P = 100% and release the return air damper to control by the SAT control loop (i.e. return air damper position is limited by the MaxRA-P endpoint, but is not directly controlled to equal MaxRA-P).</t>
+  </si>
+  <si>
+    <t>Static_pressure</t>
+  </si>
+  <si>
+    <t>SAT_Sequence</t>
+  </si>
+  <si>
+    <t>Return_fan</t>
+  </si>
+  <si>
+    <t>Relief_fan</t>
+  </si>
+  <si>
+    <t>t24_oa</t>
+  </si>
+  <si>
+    <t>62.1_oa</t>
+  </si>
+  <si>
+    <t>relief_damper_no_return_fan_static_pressure</t>
+  </si>
+  <si>
+    <t>relief_fan_building_pressure</t>
+  </si>
+  <si>
+    <t>See Section 3.1.4.5 for pressure Zone Group assignments.
+Relief fans shall be lead/lag alternated per Section 5.1.15.3.
+All operating relief fans that serve a pressure zone shall be grouped and controlled as if they were one system, running at the same speed when enabled and using the same control loop, even if they are associated with different AHUs.
+A relief fan shall be enabled when its associated supply fan is proven on, and shall be disabled otherwise.
+Building static pressure shall be time averaged with a sliding 5-minute window and 15 second sampling rate (to dampen fluctuations). The averaged value shall be that displayed and used for control.
+a.	Where multiple building pressure sensors are used, each shall be time-averaged and the highest of the averaged values for sensors within a pressure zone shall be used for control.
+A single P-only control loop for each pressure zone shall maintains the building pressure at a setpoint of 12 Pa (0.05 in. of water) with an output ranging from 0% to 100%. The loop shall be enabled when any supply fan within the pressure zone is proven ON. The loop is disabled with output set to zero otherwise.
+5.16.9.7.	Fan speed signal to all operating fans in the relief system group shall be the same and shall be equal to the PID signal but no less than the minimum speed. Except for Stage 0, discharge dampers of all relief fans shall be open only when fan is commanded ON. 
+a.	Stage 0 (barometric relief). When relief system is enabled, and the control loop output is above 5%, open the motorized dampers to all relief fans serving the relief system group that are enabled; close the dampers when the loop output drops to 0% for 5 minutes.
+b.	Stage Up. When control loop is above minimum speed plus 15%, start stage-up timer. Each time the timer reaches 7 minutes, start the next relief fan (and open the associated damper) in the relief system group, per staging order, and reset the timer to 0. The timer is reset to 0 and frozen if control loop is below minimum speed plus 15%. 
+1.	For systems where relief fans share a common relief fan inlet plenum:  When staging from Stage 0 (no relief fans) to Stage 1 (one relief fan), the relief dampers of all nonoperating relief fans must be closed.
+2.	For systems where relief fans do not share a common relief fan inlet plenum: When staging from Stage 0 (no relief fans) to Stage 1 (one relief fan), the discharge dampers of all nonoperating relief fans shall remain open when the associated supply fan is proven ON.
+c.	Stage Down. When PID loop is below minimum speed, start stage-down timer. Each time the timer reaches 5 minutes, shut off lag fan per staging order and reset the timer to 0. The timer is reset to 0 and frozen if PID loop rises above minimum speed or all fans are OFF. If all fans are OFF, go to Stage 0 (all dampers open and all fans OFF).</t>
+  </si>
+  <si>
+    <t>Control of Actuated Relief Dampers without Fans
+Relief dampers shall be enabled when the associated supply fan is proven ON, and disabled otherwise. 
+When enabled, use a P-only control loop to modulate relief dampers to maintain 12 Pa (0.05 in. of water) building static pressure. Close damper when disabled.</t>
+  </si>
+  <si>
+    <t>return_fan_building_pressure_Control</t>
+  </si>
+  <si>
+    <t>return_fan_airflow_tracking</t>
+  </si>
+  <si>
+    <t>Return-Fan Control − Direct Building Pressure
+See Section 3.1.4.5 for pressure Zone Group assignments.
+Return fan operates whenever the associated supply fan is proven ON and shall be off otherwise.
+Return fans shall be controlled to maintain return-fan discharge static pressure at setpoint (Section 5.16.10.5).
+Building static pressure shall be time averaged with a sliding 5-minute window and 15 second sampling rate (to dampen fluctuations). The averaged value shall be that displayed and used for control.
+a.	Where multiple building pressure sensors are used, the highest of the averaged values for sensors within a pressure zone shall be used for control.
+A single P-only control loop for each pressure zone shall modulate to maintain the building pressure at a setpoint of 12 Pa (0.05 in. of water) with an output ranging from 0% to 100%.  The loop shall be enabled when the supply and return fans for any unit within the pressure zone are proven ON and the minimum outdoor air damper is open.  The exhaust dampers shall be closed with loop output set to zero otherwise.  All exhaust damper and return fan static pressure setpoints for units in an associated pressure zone shall be sequenced based on building pressure control loop output signal, as shown in Figure 5.16.10.5 from ASHRAE guideline 36.
+a.	From 0% to 50%, the building pressure control loop shall modulate the exhaust dampers from 0% to 100% open.
+b.	From 51% to 100%, the building pressure control loop shall reset the return-fan discharge static pressure setpoint from RFDSPmin at 50% loop output to RFDSPmax at 100% of loop output. See Section 3.2.1.4 for RFDSPmin and RFDSPmax.</t>
+  </si>
+  <si>
+    <t>return_fan_airflow_tracking_62.1</t>
+  </si>
+  <si>
+    <t>return_fan_airflow_tracking_24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return-Fan Control − Airflow Tracking
+Return fan operates whenever associated supply fan is proven ON.
+The active differential airflow setpoint S-R-DIFF* shall be S-R-DIFF for the entire system (see Section 3.2.1.5) adjusted by the sum of the area component of the breathing zone outdoor air flow rate of zones in Zone Groups that are in Occupied Mode relative to that in all zones served by the system.
+Return-fan speed shall be controlled to maintain return airflow equal to supply airflow less differential S-R-DIFF*. Where multiple air handling units share a common return fan (i.e. dual fan dual duct), return fan speed shall be controlled to maintain return airflow equal to total supply airflow of all associated units less differential S-R-DIFF*.
+Supply fan airflow shall be limited by a reverse-acting P-only loop whose setpoint is (Vrf-max + S-R-DIFF*) and whose output is maximum supply fan speed ranging from 0% to 100%.
+Relief/exhaust dampers shall be enabled when the associated supply and return fans are proven ON and closed otherwise. Exhaust dampers shall modulate as the inverse of the return air damper per Section 5.16.2.3. Use the following euation to calculate: </t>
+  </si>
+  <si>
+    <t>〖S-R-DIFF〗^*= S-R-DIFF (∑_(all Occupied Zones)▒V_(bz-A) )/(∑_(all Zones)▒V_(bz-A) )</t>
+  </si>
+  <si>
+    <t>〖S-R-DIFF〗^*= S-R-DIFF (∑_(all Occupied Zones)▒V_(area-min) )/(∑_(all Zones)▒V_(area-min) )</t>
+  </si>
+  <si>
+    <t>alarms</t>
+  </si>
+  <si>
+    <t>Maintenance interval alarm when fan has operated for more than 1500 hours: Level 4. Reset interval count when alarm is acknowledged.
+Fan alarm is indicated by the status being different from the command for a period of 15 seconds.
+Commanded on, status off: Level 2
+Commanded off, status on: Level 4
+Filter pressure drop exceeds the larger of the alarm limit or 12.5 Pa (0.05”) for 10 minutes when airflow (expressed as a percentage of design airflow or design speed if total airflow is not known) exceeds 20%: Level 4. The alarm limit shall vary with total airflow (if available; use fan speed if total airflow is not known) as follows:
+DP_x=DP_100 (x)^1.4
+where DP100 is the high-limit pressure drop at design airflow (determine limit from filter manufacturer) and DPx is the high limit at the current airflow rate x (expressed as a fraction). For instance, the setpoint at 50% of design airflow would be (0.5)1.4, or 38% of the design high-limit pressure drop.  See Section 3.1.4.4 for DP100.
+High building pressure (more than 25 Pa [0.10 in. of water]) for 5 minutes: Level 3.
+Low building pressure (less than 0 Pa [0.0 in. of water], i.e., negative) for 5 minutes: Level 4.</t>
+  </si>
+  <si>
+    <t>Testing/Commissioning Overrides. Provide software switches that interlock to a CHW and hot-water plant level to
+a.	force HW valve full open if there is a hot-water coil,
+b.	force HW valve full closed if there is a hot-water coil,
+c.	force CHW valve full open, and
+d.	force CHW valve full closed.</t>
+  </si>
+  <si>
+    <t>freeze_protection</t>
+  </si>
+  <si>
+    <t>AFDS</t>
+  </si>
+  <si>
+    <t>Commissioning_overrides</t>
+  </si>
+  <si>
+    <t>Plant_requests</t>
+  </si>
+  <si>
+    <t>Supply Fan Start/Stop
+a.	Supply fan shall run when system is in the Cooldown Mode, Setup Mode, or Occupied Mode.
+b.	If there are any VAV-reheat boxes on perimeter zones, supply fan shall also run when system is in Setback Mode or Warmup Mode (i.e., all modes except unoccupied).
+c.	Totalize current airflow rate from VAV boxes to a software point Vps. 
+Static Pressure Set-Point Reset
+a.	Static pressure setpoint. Setpoint shall be reset using T&amp;R logic (see Section 5.1.14 from ASHRAE guideline 36) using the parameters shown in trim and respond table. 
+Static Pressure Control
+a.	Supply fan speed is controlled to maintain DSP at setpoint when the fan is proven ON. Where the Zone Groups served by the system are small, provide multiple sets of gains that are used in the control loop as a function of a load indicator (such as supply-fan airflow rate, the area of the Zone Groups that are occupied, etc.).</t>
+  </si>
+  <si>
+    <t>3.	For units with a separate minimum outdoor air damper, economizer damper minimum position MinOA-P is 0%, and return air damper maximum position MaxRA-P is modulated to control minimum outdoor air volume (see Sections related to minimum outdoor air control).</t>
+  </si>
+  <si>
+    <t>3.	For units with a single common minimum outdoor air and economizer damper, return air damper maximum position MaxRA-P and economizer damper minimum position MinOA-P are modulated to control minimum outdoor air volume (see Section 5.16.6). Economizer damper maximum position MaxOA-P is limited during minimum outdoor air control (e.g., economizer lockout due to high OAT).</t>
+  </si>
+  <si>
+    <t>1. Outdoor Airflow Setpoint for California Title 24 Ventilation
 a.	See Section 5.2.1.4 for zone outdoor air rates Zone-Abs-OA-min and Zone Des OA min.
 b.	See Section 3.1.4.2.b for setpoints AbsMinOA and DesMinOA.
 c.	Effective outdoor air absolute minimum and design minimum setpoints are recalculated continuously based on the mode of the zones being served.
@@ -799,7 +1040,7 @@
 2.	DesMinOA* is the sum of Zone-Des-OA-min for all zones in all Zone Groups that are in Occupied Mode but shall be no larger than the design minimum outdoor airflow DesMinOA.</t>
   </si>
   <si>
-    <t>Outdoor Airflow Setpoint for ASHRAE Standard 62.1-2016 Ventilation
+    <t>1. Outdoor Airflow Setpoint for ASHRAE Standard 62.1-2016 Ventilation
 a.	See Section 5.2.1.3 for zone outdoor air requirement Voz.
 b.	See Section 3.1.4.2.a for setpoints DesVou and DesVot.
 c.	The uncorrected outdoor air rate setpoint Vou is recalculated continuously based on the adjusted ventilation rates Vbz-A* and Vbz-P* of the zones being served determined in accordance with Section 5.2.1.3.
@@ -814,6 +1055,36 @@
 Ev = 1 + (Vou/Vps) – Zp
 f. Calculate the effective minimum outdoor air setpoint MinOAsp as the uncorrected outdoor air intake divided by the system ventilation efficiency, but no larger than the design total outdoor air rate DesVot:
 MinOAsp=MIN( V_ou/E_v   │  DesV_ot )</t>
+  </si>
+  <si>
+    <t>1. Outdoor Airflow Setpoint for ASHRAE Standard 62.1-2016 Ventilation
+a.	See Section above for calculation of current outdoor air setpoint MinOAsp.
+Open the minimum outdoor air damper when the supply fan is proven ON, the AHU is in Occupied Mode and MinOAsp is greater than zero.  Minimum outdoor air damper shall be closed otherwise.</t>
+  </si>
+  <si>
+    <t>1. Outdoor Airflow Setpoint for California Title 24 Ventilation
+a.	See Section above for calculation of current setpoints AbsMinOA* and DesMinOA*.
+b.	See zone CO2 control logic under terminal unit sequences.
+c.	The minimum outdoor air setpoint MinOAsp shall be reset based on the highest zone CO2 control-loop signal from AbsMinOA* at 50% signal to DesMinOA* at 100% signal.
+Open the minimum outdoor air damper when the supply fan is proven ON, the AHU is in Occupied Mode and MinOAsp is greater than zero.  Minimum outdoor air damper shall be closed otherwise.</t>
+  </si>
+  <si>
+    <t>Chilled-Water Reset Requests
+a.	If the supply air temperature exceeds the supply air temperature setpoint by 3°C (5°F) for 2 minutes, send 3 requests.
+b.	Else if the supply air temperature exceeds the supply air temperature setpoint by 2°C (3°F) for 2 minutes, send 2 requests.
+c.	Else if the CHW valve position is greater than 95%, send 1 request until the CHW valve position is less than 85%.
+d.	Else if the CHW valve position is less than 95%, send 0 requests.
+Chiller Plant Requests. Send the chiller plant that serves the system a chiller plant request as follows:
+a.	If the CHW valve position is greater than 95%, send 1 request until the CHW valve position is less than 10%.
+b.	Else if the CHW valve position is less than 95%, send 0 requests. 
+If There Is a Hot-Water Coil, Hot-Water Reset Requests
+a.	If the supply air temperature is 17°C (30°F) less than setpoint for 5 minutes, send 3 requests.
+b.	Else if the supply air temperature is 8°C (15°F) less than setpoint for 5 minutes, send 2 requests.
+c.	Else if HW valve position is greater than 95%, send 1 request until the HW valve position is less than 85%.
+d.	Else if the HW valve position is less than 95%, send 0 requests.
+If There Is a Hot-Water Coil, Heating Hot Water Plant Requests. Send the heating hot-water plant that serves the AHU a heating hot-water plant request as follows:
+a.	If the HW valve position is greater than 95%, send 1 request until the HW valve position is less than 10%.
+b.	Else if the HW valve position is less than 95%, send 0 requests.</t>
   </si>
 </sst>
 </file>
@@ -901,15 +1172,6 @@
   </cellStyles>
   <dxfs count="38">
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -932,6 +1194,15 @@
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1103,29 +1374,29 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{627E4CE9-6691-4AFC-859C-E7C0D746D35A}" name="Table6" displayName="Table6" ref="A2:G21" totalsRowShown="0" dataDxfId="13">
-  <autoFilter ref="A2:G21" xr:uid="{627E4CE9-6691-4AFC-859C-E7C0D746D35A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{627E4CE9-6691-4AFC-859C-E7C0D746D35A}" name="Table6" displayName="Table6" ref="A2:G29" totalsRowShown="0" dataDxfId="13">
+  <autoFilter ref="A2:G29" xr:uid="{627E4CE9-6691-4AFC-859C-E7C0D746D35A}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{8AE4E238-82D6-4B78-B82A-3C0A4C6B2566}" name="Required" dataDxfId="12"/>
     <tableColumn id="4" xr3:uid="{83CD2228-4A96-43E1-AE5A-FE88B5C01E71}" name="Table" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{ABA423C0-C4B9-42AC-ABAA-EBCBA72B4CB3}" name="table_column" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{88D4DF17-A024-4DE7-83C0-C7AC4C1C7FEF}" name="Section title" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{93AF809B-B0D5-4F54-9D30-110A3F3CB80F}" name="Section Applicable if" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{D441C0D1-2776-4217-AE22-160A60E2EB66}" name="Code" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{16EF8E91-9739-45BA-BC45-CC656357BCAD}" name="Sequence" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{ABA423C0-C4B9-42AC-ABAA-EBCBA72B4CB3}" name="table_column" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{88D4DF17-A024-4DE7-83C0-C7AC4C1C7FEF}" name="Section title" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{93AF809B-B0D5-4F54-9D30-110A3F3CB80F}" name="Section Applicable if" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{D441C0D1-2776-4217-AE22-160A60E2EB66}" name="Code" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{16EF8E91-9739-45BA-BC45-CC656357BCAD}" name="Sequence" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1AC01491-0428-4E65-BEB7-9A3AFE753543}" name="Trim_and_Respond_Table" displayName="Trim_and_Respond_Table" ref="A3:D14" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1AC01491-0428-4E65-BEB7-9A3AFE753543}" name="Trim_and_Respond_Table" displayName="Trim_and_Respond_Table" ref="A3:D14" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="A3:D14" xr:uid="{1AC01491-0428-4E65-BEB7-9A3AFE753543}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{475F92BB-2C46-4AA0-8A45-A52B3875DA25}" name="Variable" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{0B1D9E2C-B5E8-4405-89F2-EAB6C7034295}" name="Definition" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{9F44D363-2F18-45A8-8A15-315037E5012F}" name="Static Pressure" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{5CE867A0-EF04-4E64-9746-7BD8F7A77745}" name="Supply Air" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{475F92BB-2C46-4AA0-8A45-A52B3875DA25}" name="Variable" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{0B1D9E2C-B5E8-4405-89F2-EAB6C7034295}" name="Definition" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{9F44D363-2F18-45A8-8A15-315037E5012F}" name="Static Pressure" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{5CE867A0-EF04-4E64-9746-7BD8F7A77745}" name="Supply Air" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2952,13 +3223,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F29F9F55-D29D-4BAC-AD64-D314BD34B2FA}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" customWidth="1"/>
-    <col min="4" max="6" width="27.109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" hidden="1" customWidth="1"/>
+    <col min="2" max="3" width="22.44140625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5546875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="29.21875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="27.109375" style="3" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="160.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2982,16 +3254,16 @@
         <v>171</v>
       </c>
       <c r="C2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>214</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>215</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>153</v>
@@ -2999,53 +3271,53 @@
     </row>
     <row r="3" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>186</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>169</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>218</v>
+        <v>251</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>187</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>186</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>154</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>218</v>
+        <v>252</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -3053,18 +3325,18 @@
         <v>154</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>220</v>
+        <v>253</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -3072,13 +3344,13 @@
         <v>154</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>102</v>
+        <v>254</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3089,13 +3361,13 @@
         <v>154</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>223</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3106,13 +3378,13 @@
         <v>154</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
@@ -3124,12 +3396,14 @@
       <c r="D9" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E9" s="5"/>
+      <c r="E9" s="5" t="s">
+        <v>255</v>
+      </c>
       <c r="F9" s="5" t="s">
         <v>8</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>229</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="259.2" x14ac:dyDescent="0.3">
@@ -3141,15 +3415,17 @@
       <c r="D10" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E10" s="5"/>
+      <c r="E10" s="5" t="s">
+        <v>256</v>
+      </c>
       <c r="F10" s="5" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>159</v>
       </c>
@@ -3158,137 +3434,321 @@
       <c r="D11" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-    </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E11" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>159</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>156</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>97</v>
+        <v>239</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="E13" s="5"/>
+        <v>240</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>241</v>
+      </c>
       <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G13" s="5" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>160</v>
+        <v>239</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="E14" s="5"/>
+        <v>240</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>243</v>
+      </c>
       <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G14" s="5" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>117</v>
+        <v>159</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+        <v>157</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>117</v>
+        <v>159</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-    </row>
-    <row r="17" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
+        <v>157</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>164</v>
+        <v>239</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="D17" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>246</v>
+      </c>
       <c r="F17" s="5"/>
       <c r="G17" s="5" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="144" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>165</v>
+        <v>239</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="D18" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>245</v>
+      </c>
       <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-    </row>
-    <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G18" s="5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>219</v>
+        <v>97</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="E19" s="5"/>
+        <v>158</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>257</v>
+      </c>
       <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-    </row>
-    <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G19" s="5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>219</v>
+        <v>160</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="E20" s="5"/>
+        <v>161</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>258</v>
+      </c>
       <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G20" s="5" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>219</v>
+        <v>117</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+    </row>
+    <row r="28" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
+      <c r="E29" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5" t="s">
+        <v>283</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3329,13 +3789,13 @@
         <v>172</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>188</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -3343,7 +3803,7 @@
         <v>23</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>173</v>
@@ -3357,10 +3817,10 @@
         <v>174</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>176</v>
@@ -3371,13 +3831,13 @@
         <v>175</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -3385,13 +3845,13 @@
         <v>176</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -3399,7 +3859,7 @@
         <v>177</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>178</v>
@@ -3413,7 +3873,7 @@
         <v>179</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>180</v>
@@ -3427,7 +3887,7 @@
         <v>181</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C10" s="4">
         <v>2</v>
@@ -3441,13 +3901,13 @@
         <v>24</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>182</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -3455,13 +3915,13 @@
         <v>183</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -3469,13 +3929,13 @@
         <v>184</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -3483,13 +3943,13 @@
         <v>185</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -3501,4 +3961,68 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FF3702C-84EC-4DDB-80C3-4B27943BB77D}">
+  <dimension ref="F7:H18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="6" max="6" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="7" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="10" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="G10" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="11" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="12" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="H12" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="13" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="H13" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="14" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="H14" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="15" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="H15" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="G16" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H17" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H18" t="s">
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>